<commit_message>
Working 2026 data updates
</commit_message>
<xml_diff>
--- a/data/20241125 MeteorologicalNetworks-FERN-VF-shared.xlsx
+++ b/data/20241125 MeteorologicalNetworks-FERN-VF-shared.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jwang/Documents/projects/nbcclim/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{487EA9B3-BA19-C84E-811C-561FF789EFF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8263AF56-46BE-454F-9300-098808EDDC50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="160" yWindow="920" windowWidth="34240" windowHeight="21260" tabRatio="712" xr2:uid="{B85E001E-0A2A-45BD-9354-04487DA0E05D}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="357">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="779" uniqueCount="360">
   <si>
     <t>lat</t>
   </si>
@@ -1113,13 +1113,22 @@
   </si>
   <si>
     <t>Willow-Bowron</t>
+  </si>
+  <si>
+    <t>53.72029N</t>
+  </si>
+  <si>
+    <t>-127.25169W</t>
+  </si>
+  <si>
+    <t>IBB1 Sweeney Lake</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="26" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1293,6 +1302,18 @@
       <sz val="12"/>
       <color rgb="FF222222"/>
       <name val="Aptos"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF222222"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF222222"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="35">
@@ -2286,7 +2307,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="117">
+  <cellXfs count="119">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
@@ -2547,6 +2568,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -5629,6 +5652,23 @@
         <v>34</v>
       </c>
     </row>
+    <row r="37" spans="1:29" ht="16" x14ac:dyDescent="0.2">
+      <c r="A37" s="102" t="s">
+        <v>357</v>
+      </c>
+      <c r="B37" s="102" t="s">
+        <v>358</v>
+      </c>
+      <c r="F37" s="103" t="s">
+        <v>359</v>
+      </c>
+      <c r="H37" s="103" t="s">
+        <v>359</v>
+      </c>
+      <c r="J37" s="102">
+        <v>1146</v>
+      </c>
+    </row>
     <row r="51" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A51" s="87"/>
       <c r="B51" s="87"/>
@@ -5704,11 +5744,11 @@
   <sheetData>
     <row r="1" spans="1:7" s="14" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="13"/>
-      <c r="E1" s="105" t="s">
+      <c r="E1" s="107" t="s">
         <v>187</v>
       </c>
-      <c r="F1" s="106"/>
-      <c r="G1" s="106"/>
+      <c r="F1" s="108"/>
+      <c r="G1" s="108"/>
     </row>
     <row r="2" spans="1:7" s="21" customFormat="1" ht="33" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="15"/>
@@ -5732,7 +5772,7 @@
       </c>
     </row>
     <row r="3" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3" s="107" t="s">
+      <c r="A3" s="109" t="s">
         <v>17</v>
       </c>
       <c r="B3" s="22" t="s">
@@ -5751,7 +5791,7 @@
       <c r="G3" s="27"/>
     </row>
     <row r="4" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="108"/>
+      <c r="A4" s="110"/>
       <c r="B4" s="29" t="s">
         <v>196</v>
       </c>
@@ -5768,7 +5808,7 @@
       <c r="G4" s="34"/>
     </row>
     <row r="5" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="109"/>
+      <c r="A5" s="111"/>
       <c r="B5" s="35" t="s">
         <v>199</v>
       </c>
@@ -5803,7 +5843,7 @@
       </c>
     </row>
     <row r="7" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A7" s="107" t="s">
+      <c r="A7" s="109" t="s">
         <v>19</v>
       </c>
       <c r="B7" s="22" t="s">
@@ -5824,7 +5864,7 @@
       </c>
     </row>
     <row r="8" spans="1:7" ht="32" x14ac:dyDescent="0.2">
-      <c r="A8" s="108"/>
+      <c r="A8" s="110"/>
       <c r="B8" s="47" t="s">
         <v>207</v>
       </c>
@@ -5839,7 +5879,7 @@
       </c>
     </row>
     <row r="9" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A9" s="108"/>
+      <c r="A9" s="110"/>
       <c r="B9" s="47" t="s">
         <v>179</v>
       </c>
@@ -5854,7 +5894,7 @@
       </c>
     </row>
     <row r="10" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A10" s="108"/>
+      <c r="A10" s="110"/>
       <c r="B10" s="47" t="s">
         <v>212</v>
       </c>
@@ -5869,7 +5909,7 @@
       </c>
     </row>
     <row r="11" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A11" s="108"/>
+      <c r="A11" s="110"/>
       <c r="B11" s="47" t="s">
         <v>215</v>
       </c>
@@ -5884,7 +5924,7 @@
       </c>
     </row>
     <row r="12" spans="1:7" ht="32" x14ac:dyDescent="0.2">
-      <c r="A12" s="108"/>
+      <c r="A12" s="110"/>
       <c r="B12" s="47" t="s">
         <v>31</v>
       </c>
@@ -5899,7 +5939,7 @@
       </c>
     </row>
     <row r="13" spans="1:7" ht="32" x14ac:dyDescent="0.2">
-      <c r="A13" s="108"/>
+      <c r="A13" s="110"/>
       <c r="B13" s="53" t="s">
         <v>184</v>
       </c>
@@ -5912,7 +5952,7 @@
       <c r="G13" s="34"/>
     </row>
     <row r="14" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="109"/>
+      <c r="A14" s="111"/>
       <c r="B14" s="58" t="s">
         <v>221</v>
       </c>
@@ -5945,7 +5985,7 @@
       </c>
     </row>
     <row r="16" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A16" s="107" t="s">
+      <c r="A16" s="109" t="s">
         <v>21</v>
       </c>
       <c r="B16" s="22" t="s">
@@ -5964,7 +6004,7 @@
       <c r="G16" s="27"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A17" s="108"/>
+      <c r="A17" s="110"/>
       <c r="B17" s="29" t="s">
         <v>230</v>
       </c>
@@ -5977,7 +6017,7 @@
       <c r="G17" s="34"/>
     </row>
     <row r="18" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="109"/>
+      <c r="A18" s="111"/>
       <c r="B18" s="35" t="s">
         <v>232</v>
       </c>
@@ -6030,7 +6070,7 @@
       <c r="G20" s="69"/>
     </row>
     <row r="21" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A21" s="102" t="s">
+      <c r="A21" s="104" t="s">
         <v>24</v>
       </c>
       <c r="B21" s="70" t="s">
@@ -6048,7 +6088,7 @@
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A22" s="103"/>
+      <c r="A22" s="105"/>
       <c r="B22" s="29"/>
       <c r="C22" s="30" t="s">
         <v>243</v>
@@ -6062,7 +6102,7 @@
       </c>
     </row>
     <row r="23" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="104"/>
+      <c r="A23" s="106"/>
       <c r="B23" s="76" t="s">
         <v>185</v>
       </c>
@@ -6078,7 +6118,7 @@
       </c>
     </row>
     <row r="24" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A24" s="107" t="s">
+      <c r="A24" s="109" t="s">
         <v>25</v>
       </c>
       <c r="B24" s="22" t="s">
@@ -6097,7 +6137,7 @@
       <c r="G24" s="27"/>
     </row>
     <row r="25" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A25" s="108"/>
+      <c r="A25" s="110"/>
       <c r="B25" s="29" t="s">
         <v>63</v>
       </c>
@@ -6116,7 +6156,7 @@
       </c>
     </row>
     <row r="26" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A26" s="108"/>
+      <c r="A26" s="110"/>
       <c r="B26" s="29" t="s">
         <v>87</v>
       </c>
@@ -6133,7 +6173,7 @@
       <c r="G26" s="34"/>
     </row>
     <row r="27" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A27" s="108"/>
+      <c r="A27" s="110"/>
       <c r="B27" s="29" t="s">
         <v>35</v>
       </c>
@@ -6150,7 +6190,7 @@
       <c r="G27" s="34"/>
     </row>
     <row r="28" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="109"/>
+      <c r="A28" s="111"/>
       <c r="B28" s="35"/>
       <c r="C28" s="36" t="s">
         <v>260</v>
@@ -6167,7 +6207,7 @@
       <c r="G28" s="40"/>
     </row>
     <row r="29" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A29" s="102" t="s">
+      <c r="A29" s="104" t="s">
         <v>27</v>
       </c>
       <c r="B29" s="70" t="s">
@@ -6183,7 +6223,7 @@
       </c>
     </row>
     <row r="30" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A30" s="103"/>
+      <c r="A30" s="105"/>
       <c r="B30" s="29" t="s">
         <v>265</v>
       </c>
@@ -6197,7 +6237,7 @@
       </c>
     </row>
     <row r="31" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A31" s="103"/>
+      <c r="A31" s="105"/>
       <c r="B31" s="29" t="s">
         <v>267</v>
       </c>
@@ -6211,7 +6251,7 @@
       </c>
     </row>
     <row r="32" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A32" s="103"/>
+      <c r="A32" s="105"/>
       <c r="B32" s="29" t="s">
         <v>270</v>
       </c>
@@ -6225,7 +6265,7 @@
       </c>
     </row>
     <row r="33" spans="1:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="103"/>
+      <c r="A33" s="105"/>
       <c r="B33" s="29" t="s">
         <v>186</v>
       </c>
@@ -6268,11 +6308,11 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" s="114" t="s">
+      <c r="A2" s="116" t="s">
         <v>276</v>
       </c>
-      <c r="B2" s="115"/>
-      <c r="C2" s="112" t="s">
+      <c r="B2" s="117"/>
+      <c r="C2" s="114" t="s">
         <v>277</v>
       </c>
     </row>
@@ -6283,7 +6323,7 @@
       <c r="B3" s="2" t="s">
         <v>279</v>
       </c>
-      <c r="C3" s="113"/>
+      <c r="C3" s="115"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
@@ -6297,7 +6337,7 @@
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" s="110" t="s">
+      <c r="A5" s="112" t="s">
         <v>281</v>
       </c>
       <c r="B5" s="2" t="s">
@@ -6308,7 +6348,7 @@
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" s="111"/>
+      <c r="A6" s="113"/>
       <c r="B6" s="2" t="s">
         <v>284</v>
       </c>
@@ -6337,7 +6377,7 @@
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" s="110" t="s">
+      <c r="A9" s="112" t="s">
         <v>289</v>
       </c>
       <c r="B9" s="2" t="s">
@@ -6348,7 +6388,7 @@
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" s="116"/>
+      <c r="A10" s="118"/>
       <c r="B10" s="2" t="s">
         <v>292</v>
       </c>
@@ -6357,7 +6397,7 @@
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" s="116"/>
+      <c r="A11" s="118"/>
       <c r="B11" s="2" t="s">
         <v>294</v>
       </c>
@@ -6366,7 +6406,7 @@
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" s="111"/>
+      <c r="A12" s="113"/>
       <c r="B12" s="2" t="s">
         <v>296</v>
       </c>
@@ -6375,7 +6415,7 @@
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" s="110" t="s">
+      <c r="A13" s="112" t="s">
         <v>298</v>
       </c>
       <c r="B13" s="2" t="s">
@@ -6386,7 +6426,7 @@
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A14" s="116"/>
+      <c r="A14" s="118"/>
       <c r="B14" s="2" t="s">
         <v>301</v>
       </c>
@@ -6395,7 +6435,7 @@
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A15" s="116"/>
+      <c r="A15" s="118"/>
       <c r="B15" s="2" t="s">
         <v>303</v>
       </c>
@@ -6404,7 +6444,7 @@
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A16" s="111"/>
+      <c r="A16" s="113"/>
       <c r="B16" s="2" t="s">
         <v>123</v>
       </c>
@@ -6413,7 +6453,7 @@
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A17" s="110" t="s">
+      <c r="A17" s="112" t="s">
         <v>306</v>
       </c>
       <c r="B17" s="2" t="s">
@@ -6424,7 +6464,7 @@
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" s="116"/>
+      <c r="A18" s="118"/>
       <c r="B18" s="2" t="s">
         <v>309</v>
       </c>
@@ -6433,7 +6473,7 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A19" s="111"/>
+      <c r="A19" s="113"/>
       <c r="B19" s="2" t="s">
         <v>311</v>
       </c>
@@ -6451,7 +6491,7 @@
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A21" s="110" t="s">
+      <c r="A21" s="112" t="s">
         <v>313</v>
       </c>
       <c r="B21" s="2" t="s">
@@ -6462,7 +6502,7 @@
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A22" s="111"/>
+      <c r="A22" s="113"/>
       <c r="B22" s="2" t="s">
         <v>316</v>
       </c>

</xml_diff>

<commit_message>
Add Sweeney Lake weather station on map
</commit_message>
<xml_diff>
--- a/data/20241125 MeteorologicalNetworks-FERN-VF-shared.xlsx
+++ b/data/20241125 MeteorologicalNetworks-FERN-VF-shared.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jwang/Documents/projects/nbcclim/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8263AF56-46BE-454F-9300-098808EDDC50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F930B3AC-8A24-B440-896A-D4ECC74833ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="160" yWindow="920" windowWidth="34240" windowHeight="21260" tabRatio="712" xr2:uid="{B85E001E-0A2A-45BD-9354-04487DA0E05D}"/>
+    <workbookView xWindow="2080" yWindow="620" windowWidth="34240" windowHeight="20980" tabRatio="712" xr2:uid="{B85E001E-0A2A-45BD-9354-04487DA0E05D}"/>
   </bookViews>
   <sheets>
     <sheet name="StationList" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="779" uniqueCount="360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="777" uniqueCount="358">
   <si>
     <t>lat</t>
   </si>
@@ -1113,12 +1113,6 @@
   </si>
   <si>
     <t>Willow-Bowron</t>
-  </si>
-  <si>
-    <t>53.72029N</t>
-  </si>
-  <si>
-    <t>-127.25169W</t>
   </si>
   <si>
     <t>IBB1 Sweeney Lake</t>
@@ -5653,17 +5647,17 @@
       </c>
     </row>
     <row r="37" spans="1:29" ht="16" x14ac:dyDescent="0.2">
-      <c r="A37" s="102" t="s">
+      <c r="A37" s="102">
+        <v>53.720289999999999</v>
+      </c>
+      <c r="B37" s="102">
+        <v>-127.25169</v>
+      </c>
+      <c r="F37" s="103" t="s">
         <v>357</v>
       </c>
-      <c r="B37" s="102" t="s">
-        <v>358</v>
-      </c>
-      <c r="F37" s="103" t="s">
-        <v>359</v>
-      </c>
       <c r="H37" s="103" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="J37" s="102">
         <v>1146</v>
@@ -6818,6 +6812,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="d50a919c-bd16-47eb-b143-2d77304b7540" xsi:nil="true"/>
@@ -6826,15 +6829,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6857,6 +6851,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC9A7C8A-0EB9-48A7-B767-FF76BC2EB741}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA26F111-2A86-4A89-80A1-F8E203F45C13}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -6865,12 +6867,4 @@
     <ds:schemaRef ds:uri="359b0286-d67e-4431-ab6a-a264c3167115"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC9A7C8A-0EB9-48A7-B767-FF76BC2EB741}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>